<commit_message>
Update the verified example audit pack
</commit_message>
<xml_diff>
--- a/downloads/IFRS-Connect-Example-Audit-Pack.xlsx
+++ b/downloads/IFRS-Connect-Example-Audit-Pack.xlsx
@@ -1725,7 +1725,7 @@
     <t>FX translation</t>
   </si>
   <si>
-    <t>No presentation-currency translation was requested for this lease. Amounts remain in the lease currency shown on Inputs.</t>
+    <t>No functional-currency schedule snapshot was requested for this lease. Amounts remain in the lease currency shown on Inputs.</t>
   </si>
   <si>
     <t>Summary metric</t>
@@ -3189,7 +3189,7 @@
     <t>Deterministic content hash (SHA-256)</t>
   </si>
   <si>
-    <t>452b9003e918981bc00a365b8f031d620ed262b323897e7f2bde72c13e120fae</t>
+    <t>b0e171cd9f9ff79c0c908a1898fe2874111dbe4a6fc937051143ab39a22ddc5a</t>
   </si>
   <si>
     <t>Key inputs</t>

</xml_diff>

<commit_message>
Update the example audit pack and release notes
</commit_message>
<xml_diff>
--- a/downloads/IFRS-Connect-Example-Audit-Pack.xlsx
+++ b/downloads/IFRS-Connect-Example-Audit-Pack.xlsx
@@ -2424,7 +2424,7 @@
     <t>Journal accrual law (one interest accrual row per displayed schedule period)</t>
   </si>
   <si>
-    <t>For each displayed lease period, require exactly one recurring Accrual journal row dated on that displayed period date, with period interest and depreciation equal to the displayed liability and ROU schedules; PASS only when every period matches and no orphan accrual rows remain.</t>
+    <t>For each canonical calculation period, require exactly one recurring Accrual journal row dated on that period date, with interest and depreciation equal to the calculation's liability and ROU rows. Where the main schedules combine internal splits, Calculation rows identifies these original periods. PASS only when every calculation period matches and no orphan accrual rows remain.</t>
   </si>
   <si>
     <t>JournalInterestRows=72 SchedulePeriods=72 InterestRowsPerPeriodMax=1 InterestRowDeficitOrSurplus=0 MissingPeriods=0 DuplicatePeriods=0 DateMismatches=0 FirstCountMismatchPeriod=n/a FirstDateMismatchPeriod=n/a OrphanPeriods=0 OrphanJournalDates=none MaxPerPeriodInterestDiff=0 MaxInterestDiffPeriod=n/a MaxPerPeriodInterestPnlDiff=0 MaxInterestPnlDiffPeriod=n/a MaxPerPeriodDepDiff=0 MaxDepDiffPeriod=n/a MaxPerPeriodAccumDepDiff=0 MaxAccumDepDiffPeriod=n/a TotalInterestDiff=0 TotalInterestPnlDiff=0</t>
@@ -2694,7 +2694,7 @@
     <t>Accrual row count delta = 0, rows per period = 1, date mismatches = 0, and no tolerance on the amounts: canonical interest and depreciation must match exactly.</t>
   </si>
   <si>
-    <t>Recurring accrual journals no longer reconcile one-to-one with displayed schedule periods, so period evidence is not safe to report.</t>
+    <t>Recurring accrual journals no longer reconcile one-to-one with the original calculation periods listed under Calculation rows, so period evidence is not safe to report.</t>
   </si>
   <si>
     <t>Scope events checked &gt; 0 implies carry mismatches = 0, unexpected same-day scope remeasure rows = 0 and missing follow-on events = 0; scope events proportion checked &gt; 0 implies proportion mismatches = 0</t>
@@ -3033,7 +3033,7 @@
     <t>Engine version</t>
   </si>
   <si>
-    <t>2026-09-04-free-preview-keeps-full-depreciation-total-v1</t>
+    <t>2026-09-09-original-period-display-provenance-v1</t>
   </si>
   <si>
     <t>Result generated UTC</t>
@@ -3048,7 +3048,7 @@
     <t>Schedule JSON checksum (SHA-256)</t>
   </si>
   <si>
-    <t>3d045e8e619d99fd3d77a36ac509caa66204fc7d3ae417b799a3a66484b2f876</t>
+    <t>b4241ca3ed1c4dd6fa1a273d9f45290e9e5f18b67ac472a44a29d736075e6731</t>
   </si>
   <si>
     <t>Run certificate version</t>
@@ -3084,7 +3084,7 @@
     <t>Manifest hash (SHA-256)</t>
   </si>
   <si>
-    <t>26bad7ce074550e0eb177cd685ef914fbf02e21bca08c3630574fed924b02de2</t>
+    <t>d4b143e1624fe9f8d6c0ec44bb81197c18918d438538cb2d89f5b271821808da</t>
   </si>
   <si>
     <t>Liability rows</t>
@@ -3189,7 +3189,7 @@
     <t>Deterministic content hash (SHA-256)</t>
   </si>
   <si>
-    <t>b0e171cd9f9ff79c0c908a1898fe2874111dbe4a6fc937051143ab39a22ddc5a</t>
+    <t>ce239bbf0b17d6359907073b9255b5aa6b8aa18f0689f074dcea9658fdbdad5e</t>
   </si>
   <si>
     <t>Key inputs</t>
@@ -27250,7 +27250,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="16" ht="68" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" ht="100" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="36" t="s">
         <v>784</v>
       </c>
@@ -29719,7 +29719,7 @@
         <v>992</v>
       </c>
       <c r="B9" s="21">
-        <v>389299</v>
+        <v>389618</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Refresh the example audit pack and release history
</commit_message>
<xml_diff>
--- a/downloads/IFRS-Connect-Example-Audit-Pack.xlsx
+++ b/downloads/IFRS-Connect-Example-Audit-Pack.xlsx
@@ -3033,7 +3033,7 @@
     <t>Engine version</t>
   </si>
   <si>
-    <t>2026-09-09-original-period-display-provenance-v1</t>
+    <t>2026-09-10-paid-lease-name-preservation-v1</t>
   </si>
   <si>
     <t>Result generated UTC</t>
@@ -3048,7 +3048,7 @@
     <t>Schedule JSON checksum (SHA-256)</t>
   </si>
   <si>
-    <t>b4241ca3ed1c4dd6fa1a273d9f45290e9e5f18b67ac472a44a29d736075e6731</t>
+    <t>af65a7eb1d36eb44b625c708200b84e9050432f43194372c278697ce083f9733</t>
   </si>
   <si>
     <t>Run certificate version</t>
@@ -3084,7 +3084,7 @@
     <t>Manifest hash (SHA-256)</t>
   </si>
   <si>
-    <t>d4b143e1624fe9f8d6c0ec44bb81197c18918d438538cb2d89f5b271821808da</t>
+    <t>a33a69da397db17939d459730806a683af6325c4d08d4afed48d6e9015ba85d0</t>
   </si>
   <si>
     <t>Liability rows</t>
@@ -3189,7 +3189,7 @@
     <t>Deterministic content hash (SHA-256)</t>
   </si>
   <si>
-    <t>ce239bbf0b17d6359907073b9255b5aa6b8aa18f0689f074dcea9658fdbdad5e</t>
+    <t>0e07affc493749f0a2a6ae00b341b70c9ab24642e30d25498cbdc6efcded008b</t>
   </si>
   <si>
     <t>Key inputs</t>
@@ -29719,7 +29719,7 @@
         <v>992</v>
       </c>
       <c r="B9" s="21">
-        <v>389618</v>
+        <v>389600</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>